<commit_message>
--User changes  -Add post_smartcrop.
--Bug fixes
 -Fix bug in crackle.
 -Wrong point assignment in hexaplay3D, hexnix3D.
 -Improper Z assignment in rblur.
 -Fix inconsistency with original in circlecrop.
 -Put EMBER_ROOT bakc to ./../../../ in default.pri. This is TBD.

--Code changes
 -Convert all enums to class enum to be consistent with C++11 style.
 -Convert some if/else statements in filter classes to case statements.
 -Add overloaded stream operators to print various enums.
 -Optimize crob, nBlur.
 -Fix weird assignment statement in falloff3.
 -Cleanup in VarFuncs::SimplexNoise3D().
 -Replace fabs() with std::abs().
 -General cleanup.
</commit_message>
<xml_diff>
--- a/Data/Variations.xlsx
+++ b/Data/Variations.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="574">
   <si>
     <t>flatten</t>
   </si>
@@ -1734,6 +1734,9 @@
   </si>
   <si>
     <t>crackle</t>
+  </si>
+  <si>
+    <t>smartshape</t>
   </si>
 </sst>
 </file>
@@ -3690,11 +3693,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="108275712"/>
-        <c:axId val="89839232"/>
+        <c:axId val="40138752"/>
+        <c:axId val="108909632"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="108275712"/>
+        <c:axId val="40138752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3703,7 +3706,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="89839232"/>
+        <c:crossAx val="108909632"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3711,7 +3714,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89839232"/>
+        <c:axId val="108909632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3722,7 +3725,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="108275712"/>
+        <c:crossAx val="40138752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4065,7 +4068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I314"/>
+  <dimension ref="A1:I298"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48" bestFit="1" customWidth="1"/>
@@ -4277,8 +4280,8 @@
       <c r="E14" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>420</v>
+      <c r="G14" s="3" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4292,7 +4295,7 @@
         <v>110</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>567</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4362,6 +4365,9 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="E22" s="4" t="s">
         <v>117</v>
       </c>
@@ -4370,8 +4376,8 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>13</v>
+      <c r="A23" s="2" t="s">
+        <v>393</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>118</v>
@@ -4381,8 +4387,8 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>393</v>
+      <c r="A24" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>119</v>
@@ -4392,32 +4398,32 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>51</v>
+      <c r="A25" s="2" t="s">
+        <v>239</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>239</v>
+      <c r="A26" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>52</v>
+      <c r="A27" s="2" t="s">
+        <v>233</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>233</v>
+      <c r="A28" s="3" t="s">
+        <v>246</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>123</v>
@@ -4425,7 +4431,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>246</v>
+        <v>304</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>124</v>
@@ -4433,7 +4439,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>304</v>
+        <v>279</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>125</v>
@@ -4441,7 +4447,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>126</v>
@@ -4449,7 +4455,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>127</v>
@@ -4457,23 +4463,23 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>280</v>
+        <v>53</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>53</v>
+      <c r="A34" s="5" t="s">
+        <v>270</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
-        <v>270</v>
+      <c r="A35" s="3" t="s">
+        <v>273</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>130</v>
@@ -4481,15 +4487,15 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>256</v>
+      <c r="A37" s="2" t="s">
+        <v>235</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>132</v>
@@ -4497,15 +4503,15 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>234</v>
+      <c r="A39" s="3" t="s">
+        <v>377</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>134</v>
@@ -4513,7 +4519,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>135</v>
@@ -4521,7 +4527,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>376</v>
+        <v>54</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>136</v>
@@ -4529,7 +4535,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>54</v>
+        <v>379</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>137</v>
@@ -4537,7 +4543,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>138</v>
@@ -4545,23 +4551,23 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>378</v>
+        <v>55</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>55</v>
+      <c r="A45" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>56</v>
+      <c r="A46" s="3" t="s">
+        <v>197</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>141</v>
@@ -4569,20 +4575,23 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>197</v>
+        <v>94</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="E48" s="4" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>94</v>
+        <v>381</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>144</v>
@@ -4590,15 +4599,15 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>247</v>
+        <v>380</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
-        <v>381</v>
+      <c r="A51" s="2" t="s">
+        <v>389</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>146</v>
@@ -4606,15 +4615,15 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
-        <v>389</v>
+      <c r="A53" s="3" t="s">
+        <v>349</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>148</v>
@@ -4622,7 +4631,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>348</v>
+        <v>16</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>149</v>
@@ -4630,7 +4639,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>349</v>
+        <v>383</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>150</v>
@@ -4638,7 +4647,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>151</v>
@@ -4646,7 +4655,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>383</v>
+        <v>198</v>
       </c>
       <c r="E57" s="4" t="s">
         <v>152</v>
@@ -4654,39 +4663,39 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>57</v>
+        <v>350</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
-        <v>198</v>
+      <c r="A59" s="2" t="s">
+        <v>242</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>350</v>
+      <c r="A60" s="2" t="s">
+        <v>327</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
-        <v>242</v>
+      <c r="A61" s="3" t="s">
+        <v>257</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>327</v>
+      <c r="A62" s="3" t="s">
+        <v>258</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>157</v>
@@ -4694,7 +4703,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>158</v>
@@ -4702,7 +4711,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>159</v>
@@ -4710,7 +4719,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E65" s="4" t="s">
         <v>160</v>
@@ -4718,7 +4727,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>260</v>
+        <v>199</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>161</v>
@@ -4726,7 +4735,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>261</v>
+        <v>12</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>162</v>
@@ -4734,15 +4743,15 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>199</v>
+        <v>262</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
-        <v>12</v>
+      <c r="A69" s="2" t="s">
+        <v>390</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>164</v>
@@ -4750,15 +4759,15 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="2" t="s">
-        <v>390</v>
+      <c r="A71" s="3" t="s">
+        <v>264</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>166</v>
@@ -4766,7 +4775,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>263</v>
+        <v>382</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>167</v>
@@ -4774,7 +4783,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>168</v>
@@ -4782,7 +4791,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>382</v>
+        <v>58</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>169</v>
@@ -4790,7 +4799,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>265</v>
+        <v>59</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>170</v>
@@ -4798,7 +4807,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>58</v>
+        <v>424</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>171</v>
@@ -4806,7 +4815,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>172</v>
@@ -4814,7 +4823,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>424</v>
+        <v>299</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>173</v>
@@ -4822,7 +4831,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>20</v>
+        <v>367</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>174</v>
@@ -4830,39 +4839,39 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>299</v>
+        <v>60</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="3" t="s">
-        <v>367</v>
+      <c r="A81" s="5" t="s">
+        <v>61</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="3" t="s">
-        <v>60</v>
+      <c r="A82" s="5" t="s">
+        <v>411</v>
       </c>
       <c r="E82" s="4" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="5" t="s">
-        <v>61</v>
+      <c r="A83" s="3" t="s">
+        <v>0</v>
       </c>
       <c r="E83" s="4" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="5" t="s">
-        <v>411</v>
+      <c r="A84" s="3" t="s">
+        <v>266</v>
       </c>
       <c r="E84" s="4" t="s">
         <v>179</v>
@@ -4870,7 +4879,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>0</v>
+        <v>267</v>
       </c>
       <c r="E85" s="4" t="s">
         <v>180</v>
@@ -4878,63 +4887,63 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>266</v>
+        <v>351</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="3" t="s">
-        <v>267</v>
+      <c r="A87" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="E87" s="4" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="3" t="s">
-        <v>351</v>
+      <c r="A88" s="5" t="s">
+        <v>288</v>
       </c>
       <c r="E88" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
-        <v>236</v>
+      <c r="A89" s="3" t="s">
+        <v>200</v>
       </c>
       <c r="E89" s="4" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="5" t="s">
-        <v>288</v>
+      <c r="A90" s="2" t="s">
+        <v>391</v>
       </c>
       <c r="E90" s="4" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="3" t="s">
-        <v>200</v>
+      <c r="A91" s="2" t="s">
+        <v>394</v>
       </c>
       <c r="E91" s="4" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="2" t="s">
-        <v>391</v>
+      <c r="A92" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E92" s="4" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
-        <v>394</v>
+      <c r="A93" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E93" s="4" t="s">
         <v>188</v>
@@ -4942,7 +4951,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>62</v>
+        <v>201</v>
       </c>
       <c r="E94" s="4" t="s">
         <v>189</v>
@@ -4950,7 +4959,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>63</v>
+        <v>202</v>
       </c>
       <c r="E95" s="4" t="s">
         <v>190</v>
@@ -4958,7 +4967,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E96" s="4" t="s">
         <v>191</v>
@@ -4966,7 +4975,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>202</v>
+        <v>64</v>
       </c>
       <c r="E97" s="4" t="s">
         <v>192</v>
@@ -4974,7 +4983,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>203</v>
+        <v>462</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>193</v>
@@ -4982,1009 +4991,1004 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>64</v>
+        <v>204</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>194</v>
       </c>
     </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="3" t="s">
-        <v>462</v>
+      <c r="A102" s="2" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>204</v>
+        <v>66</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>65</v>
+        <v>407</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="2" t="s">
-        <v>237</v>
+      <c r="A105" s="3" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="2" t="s">
-        <v>395</v>
+      <c r="A106" s="5" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>66</v>
+      <c r="A107" s="5" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
-        <v>407</v>
+      <c r="A108" s="5" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
-        <v>408</v>
+      <c r="A109" s="2" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="5" t="s">
-        <v>412</v>
+      <c r="A110" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="5" t="s">
-        <v>413</v>
+      <c r="A111" s="2" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="5" t="s">
-        <v>414</v>
+      <c r="A112" s="2" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>328</v>
+        <v>356</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" s="3" t="s">
-        <v>67</v>
+      <c r="A114" s="2" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" s="2" t="s">
-        <v>356</v>
+      <c r="A117" s="3" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>357</v>
+        <v>386</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" s="2" t="s">
-        <v>358</v>
+      <c r="A119" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="2" t="s">
-        <v>359</v>
+      <c r="A120" s="3" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>368</v>
+        <v>15</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" s="2" t="s">
-        <v>386</v>
+      <c r="A122" s="3" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" s="3" t="s">
-        <v>14</v>
+      <c r="A123" s="2" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>415</v>
+        <v>68</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>15</v>
+        <v>251</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>205</v>
+        <v>303</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A127" s="2" t="s">
-        <v>423</v>
+      <c r="A127" s="3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>68</v>
+        <v>238</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A129" s="3" t="s">
-        <v>251</v>
+      <c r="A129" s="2" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>303</v>
+        <v>268</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>69</v>
+        <v>418</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>238</v>
+        <v>206</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
-        <v>329</v>
+      <c r="A133" s="3" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
-        <v>268</v>
+        <v>417</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" s="3" t="s">
-        <v>418</v>
+      <c r="A135" s="2" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" s="3" t="s">
-        <v>206</v>
+      <c r="A136" s="2" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="3" t="s">
-        <v>416</v>
+      <c r="A137" s="2" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
-        <v>417</v>
+        <v>207</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
-        <v>330</v>
+      <c r="A139" s="3" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A140" s="2" t="s">
-        <v>331</v>
+      <c r="A140" s="3" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>332</v>
+        <v>396</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="3" t="s">
-        <v>207</v>
+      <c r="A142" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="3" t="s">
-        <v>360</v>
+      <c r="A143" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
-        <v>373</v>
+        <v>403</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>396</v>
+        <v>334</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A148" s="2" t="s">
-        <v>208</v>
+      <c r="A148" s="3" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A149" s="2" t="s">
-        <v>397</v>
+      <c r="A149" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
-        <v>232</v>
+        <v>293</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A151" s="2" t="s">
-        <v>333</v>
+      <c r="A151" s="3" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
-        <v>403</v>
+        <v>70</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" s="2" t="s">
-        <v>334</v>
+      <c r="A153" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" s="3" t="s">
-        <v>365</v>
+      <c r="A154" s="2" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" s="3" t="s">
-        <v>21</v>
+      <c r="A155" s="2" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
-        <v>293</v>
+        <v>72</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
-        <v>281</v>
+        <v>209</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" s="3" t="s">
-        <v>71</v>
+      <c r="A159" s="2" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" s="3" t="s">
-        <v>72</v>
+      <c r="A163" s="2" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" s="3" t="s">
-        <v>209</v>
+      <c r="A164" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165" s="2" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" s="3" t="s">
-        <v>73</v>
+      <c r="A166" s="2" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" s="2" t="s">
-        <v>337</v>
+      <c r="A167" s="3" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" s="2" t="s">
-        <v>338</v>
+      <c r="A168" s="3" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" s="2" t="s">
-        <v>340</v>
+      <c r="A170" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" s="2" t="s">
-        <v>341</v>
+      <c r="A171" s="3" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A172" s="2" t="s">
-        <v>342</v>
+      <c r="A172" s="3" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" s="2" t="s">
-        <v>343</v>
+      <c r="A173" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A174" s="2" t="s">
-        <v>344</v>
+      <c r="A174" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="s">
-        <v>210</v>
+        <v>76</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="s">
-        <v>211</v>
+        <v>361</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A177" s="2" t="s">
-        <v>345</v>
+      <c r="A177" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
-        <v>212</v>
+        <v>31</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
-        <v>292</v>
+        <v>29</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
-        <v>419</v>
+        <v>30</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
-        <v>75</v>
+        <v>426</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
-        <v>76</v>
+        <v>32</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
-        <v>361</v>
+        <v>301</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
-        <v>28</v>
+        <v>291</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
-        <v>31</v>
+        <v>78</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
-        <v>30</v>
+        <v>80</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
-        <v>426</v>
+        <v>82</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
-        <v>301</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A193" s="3" t="s">
-        <v>291</v>
+      <c r="A193" s="5" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A194" s="3" t="s">
-        <v>78</v>
+      <c r="A194" s="2" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
-        <v>79</v>
+        <v>213</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="3" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A198" s="3" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" s="3" t="s">
-        <v>9</v>
+        <v>306</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" s="5" t="s">
-        <v>400</v>
+        <v>425</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A202" s="2" t="s">
-        <v>249</v>
+      <c r="A202" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" s="3" t="s">
-        <v>213</v>
+        <v>300</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" s="3" t="s">
-        <v>83</v>
+        <v>290</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" s="3" t="s">
-        <v>25</v>
+        <v>214</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" s="3" t="s">
-        <v>26</v>
+        <v>215</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" s="3" t="s">
-        <v>306</v>
+        <v>5</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" s="3" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A209" s="5" t="s">
-        <v>425</v>
+        <v>399</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A210" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A211" s="3" t="s">
-        <v>300</v>
+        <v>22</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A212" s="3" t="s">
-        <v>290</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A213" s="3" t="s">
-        <v>214</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A214" s="3" t="s">
-        <v>215</v>
+        <v>84</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A215" s="3" t="s">
-        <v>5</v>
+        <v>384</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A216" s="3" t="s">
-        <v>6</v>
+      <c r="A216" s="2" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A217" s="5" t="s">
-        <v>399</v>
+      <c r="A217" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A218" s="3" t="s">
-        <v>23</v>
+      <c r="A218" s="2" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A219" s="3" t="s">
-        <v>22</v>
+      <c r="A219" s="2" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A220" s="3" t="s">
-        <v>3</v>
+      <c r="A220" s="2" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A221" s="3" t="s">
-        <v>4</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222" s="3" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A223" s="3" t="s">
-        <v>84</v>
+      <c r="A223" s="2" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A224" s="3" t="s">
-        <v>384</v>
+        <v>217</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A225" s="2" t="s">
-        <v>346</v>
+      <c r="A225" s="3" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A226" s="3" t="s">
-        <v>85</v>
+        <v>363</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A227" s="2" t="s">
-        <v>240</v>
+      <c r="A227" s="3" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A228" s="2" t="s">
-        <v>241</v>
+      <c r="A228" s="3" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A229" s="2" t="s">
-        <v>325</v>
+      <c r="A229" s="3" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A230" s="3" t="s">
-        <v>86</v>
+        <v>248</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A231" s="3" t="s">
-        <v>216</v>
+        <v>87</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A232" s="2" t="s">
-        <v>324</v>
+      <c r="A232" s="3" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A233" s="3" t="s">
-        <v>217</v>
+      <c r="A233" s="2" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
-        <v>372</v>
+        <v>302</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
-        <v>371</v>
+        <v>88</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A238" s="3" t="s">
-        <v>421</v>
+        <v>218</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A239" s="3" t="s">
-        <v>248</v>
+      <c r="A239" s="2" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A240" s="3" t="s">
-        <v>87</v>
+      <c r="A240" s="2" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A241" s="3" t="s">
-        <v>245</v>
+      <c r="A241" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A243" s="3" t="s">
-        <v>370</v>
+      <c r="A243" s="2" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A244" s="3" t="s">
-        <v>369</v>
+      <c r="A244" s="2" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A245" s="3" t="s">
-        <v>302</v>
+      <c r="A245" s="2" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A246" s="3" t="s">
-        <v>88</v>
+      <c r="A246" s="2" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A247" s="3" t="s">
-        <v>218</v>
+      <c r="A247" s="2" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A248" s="2" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A249" s="2" t="s">
-        <v>310</v>
+      <c r="A249" s="3" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A250" s="2" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A251" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A252" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A253" s="2" t="s">
-        <v>316</v>
+      <c r="A253" s="3" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A254" s="2" t="s">
-        <v>317</v>
+      <c r="A254" s="3" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A255" s="2" t="s">
-        <v>318</v>
+      <c r="A255" s="3" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
-        <v>219</v>
+        <v>398</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A258" s="2" t="s">
-        <v>320</v>
+      <c r="A258" s="3" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A259" s="2" t="s">
-        <v>321</v>
+      <c r="A259" s="3" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A260" s="2" t="s">
-        <v>322</v>
+      <c r="A260" s="3" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A261" s="3" t="s">
-        <v>231</v>
+      <c r="A261" s="2" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A262" s="3" t="s">
-        <v>366</v>
+      <c r="A262" s="2" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
-        <v>287</v>
+        <v>323</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
-        <v>326</v>
+        <v>295</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
-        <v>398</v>
+        <v>271</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A266" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
-        <v>221</v>
+        <v>272</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A268" s="3" t="s">
-        <v>404</v>
+        <v>223</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A270" s="2" t="s">
-        <v>296</v>
+      <c r="A270" s="3" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A271" s="3" t="s">
-        <v>323</v>
+      <c r="A271" s="2" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A272" s="2" t="s">
-        <v>295</v>
+      <c r="A272" s="3" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A273" s="3" t="s">
-        <v>271</v>
+        <v>224</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A274" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A275" s="3" t="s">
-        <v>272</v>
+        <v>226</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A276" s="3" t="s">
-        <v>223</v>
+        <v>375</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A277" s="2" t="s">
-        <v>297</v>
+      <c r="A277" s="3" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A278" s="3" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A279" s="2" t="s">
-        <v>298</v>
+      <c r="A279" s="5" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A280" s="3" t="s">
-        <v>89</v>
+      <c r="A280" s="2" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A281" s="3" t="s">
-        <v>224</v>
+        <v>406</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A282" s="3" t="s">
-        <v>225</v>
+      <c r="A282" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A285" s="3" t="s">
-        <v>226</v>
+      <c r="A285" s="2" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A286" s="3" t="s">
-        <v>375</v>
+        <v>95</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A287" s="3" t="s">
-        <v>374</v>
+        <v>282</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A288" s="3" t="s">
-        <v>269</v>
+        <v>230</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A289" s="5" t="s">
-        <v>227</v>
+      <c r="A289" s="3" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A290" s="2" t="s">
-        <v>312</v>
+      <c r="A290" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291" s="3" t="s">
+        <v>405</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A292" s="3" t="s">
-        <v>406</v>
+        <v>92</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
-        <v>243</v>
+        <v>347</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A294" s="3" t="s">
-        <v>229</v>
+        <v>93</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A295" s="3" t="s">
-        <v>90</v>
+      <c r="A295" s="5" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A296" s="2" t="s">
-        <v>313</v>
+      <c r="A296" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A297" s="3" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A298" s="3" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A300" s="3" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A301" s="3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A303" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A304" s="3" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A306" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A307" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A308" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A311" s="5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A312" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A313" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A314" s="3" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>